<commit_message>
Clean public source-data process traces
</commit_message>
<xml_diff>
--- a/manuscript_package/supplementary_tables/HistoSet_supplementary_tables_publication.xlsx
+++ b/manuscript_package/supplementary_tables/HistoSet_supplementary_tables_publication.xlsx
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>work/histoset/scripts/prepare_histoset_fullscale_512.py</t>
+          <t>tensor preparation script</t>
         </is>
       </c>
     </row>
@@ -5265,8 +5265,6 @@
           <t>4 - glomeruloid glands</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5297,8 +5295,6 @@
           <t>4 - glomeruloid glands</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5819,7 +5815,6 @@
           <t>prepared_samples</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5832,7 +5827,6 @@
           <t>preprocess_errors</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>pass</t>
@@ -5845,7 +5839,6 @@
           <t>train_samples</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>recorded</t>
@@ -5858,7 +5851,6 @@
           <t>val_samples</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>recorded</t>
@@ -5871,7 +5863,6 @@
           <t>test_samples</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>recorded</t>

</xml_diff>